<commit_message>
Started development of the Streamlit-based front-end portion of the project along with further dissemination of model evaluation results.
</commit_message>
<xml_diff>
--- a/dissemination/Brain Tumor Classification Model Comparisons Metrics.xlsx
+++ b/dissemination/Brain Tumor Classification Model Comparisons Metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cochr\Data Science Projects\Brain-Tumor-Detection\dissemination\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363420C5-2E30-4089-AD16-74F2FD094105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{087408AD-58C6-4007-9412-93FF4B5BC4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{886F016B-F3B6-4904-9251-B24D56E16486}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
   <si>
     <t>Epoch Size</t>
   </si>
@@ -54,6 +54,15 @@
   </si>
   <si>
     <t>1x10-6</t>
+  </si>
+  <si>
+    <t>Var</t>
+  </si>
+  <si>
+    <t>RLROP</t>
+  </si>
+  <si>
+    <t>RLROP + ES</t>
   </si>
 </sst>
 </file>
@@ -141,13 +150,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -165,6 +173,92 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>28574</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07383DF9-2E04-4781-0758-B661372606B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1847850" y="4410074"/>
+          <a:ext cx="2809875" cy="1876425"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" u="sng"/>
+            <a:t>ES</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" u="sng" baseline="0"/>
+            <a:t> + RLROP Notes:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="171450" indent="-171450">
+            <a:buFont typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:buChar char="•"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -484,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{157E6442-83B2-458A-A7D7-44481521E105}">
-  <dimension ref="D4:K12"/>
+  <dimension ref="D4:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="11.5703125" customWidth="1"/>
@@ -624,12 +718,41 @@
       <c r="K11" s="3"/>
     </row>
     <row r="12" spans="4:11" x14ac:dyDescent="0.25">
-      <c r="J12" s="5">
+      <c r="J12" s="4">
         <v>200</v>
       </c>
       <c r="K12" s="4"/>
+    </row>
+    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="D21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>